<commit_message>
Add Incoming Official Documents Management module
</commit_message>
<xml_diff>
--- a/OUTPUT/DATA_TIEN_DO_KPI.xlsx
+++ b/OUTPUT/DATA_TIEN_DO_KPI.xlsx
@@ -8,6 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GANTT_KHDT" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VAN_BAN_DEN" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -572,7 +574,6 @@
           <t>Có vướng mắc</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>Khách thuê (Bà Hằng) đang gặp khó khăn tài chính, đề xuất phương án cấn trừ tài sản cố định hoặc khởi kiện nếu không hợp tác thanh toán trước 30/06.</t>
@@ -653,8 +654,6 @@
           <t>Đang thực hiện</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr">
         <is>
           <t>2026-05-15 11:00:00</t>
@@ -730,11 +729,424 @@
           <t>Đang thực hiện</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr">
         <is>
           <t>2026-07-23 08:30:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TenDuAn</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>TenCongViec</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>GiaiDoan</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>NgayBatDau</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>NgayKetThuc</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>PhanTramHoanThanh</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>NgayCapNhat</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GNT-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Dự án Xây dựng Khu Đô thị Marina</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Khảo sát thị trường &amp; Khả thi</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1. Chuẩn bị Đầu tư &amp; Nghiên cứu Tiền khả thi</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-07-24 13:56:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GNT-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Dự án Xây dựng Khu Đô thị Marina</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Thiết kế quy hoạch &amp; Kiến trúc</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2. Pháp lý Dự án &amp; Quy hoạch 1/500</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>80</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-07-24 13:56:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GNT-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Dự án Xây dựng Khu Đô thị Marina</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Phê duyệt Pháp lý &amp; Báo cáo KHĐT</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2. Pháp lý Dự án &amp; Quy hoạch 1/500</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Mốc 1: Phê duyệt Pháp lý &amp; GPXD</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-07-24 13:56:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GNT-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Dự án Xây dựng Khu Đô thị Marina</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Báo cáo Nghiên cứu Tiền khả thi</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1. Chuẩn bị Đầu tư &amp; Nghiên cứu Tiền khả thi</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>40</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-07-24 13:56:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GNT-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Dự án Xây dựng Khu Đô thị Marina</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Trình duyệt Thẩm định Đầu tư</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>4. Thiết kế Bản vẽ Thi công &amp; Thẩm định</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Mốc 2: Cất nóc công trình</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-07-24 13:56:13</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>DonVi</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>SoKyHieu</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>NgayBanHanh</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>CoQuanGui</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>TrichYeu</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>TenDuAn</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>GanttTaskId</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>BanChuTri</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>LinkFile</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>TrangThai</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>NgayCapNhat</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DOC-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CTY CP ĐẦU TƯ ĐÀ NẴNG - MIỀN TRUNG</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>DMT-2026-001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SSo Quy hoach Kien truc</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Van ban huong dan quy hoach du an Khu do thi Phuoc Ly</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>KĐT Phước Lý &amp; Phước Lý MR</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Ban Kế hoạch Đầu tư</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/example-doc-123</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>⏳ Đang xử lý</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-07-24 14:05:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Filter incoming documents with completion deadlines and auto-trigger overdue alerts
</commit_message>
<xml_diff>
--- a/OUTPUT/DATA_TIEN_DO_KPI.xlsx
+++ b/OUTPUT/DATA_TIEN_DO_KPI.xlsx
@@ -1017,7 +1017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1150,6 +1150,133 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DOC-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CTY CP ĐẦU TƯ ĐÀ NẴNG - MIỀN TRUNG</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DMT-2026-001CV-2026-X1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>So Tai nguyen va Moi truong</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Cong van ra soat du an Phuoc Ly</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>KĐT Phước Lý &amp; Phước Lý MR</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Ban Kế hoạch Đầu tư</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/examhttps://drive.google.com/test-doc-x1ple-doc-123</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>⏳ Đang xử lý</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-07-24 14:25:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DOC-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CTY CP XÂY DỰNG CÔNG TRÌNH GIAO THÔNG ĐN-MT</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DMT-2026-001CV-2026-X1CV-2026-X2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>So Tai nguyen va Moi truongSSo Xay dung TP. Da Nang</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Cong van ra soat du an PhuCong van nghiem thu ban giao truc I Tay Bac
+oc Ly</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Trục I Tây Bắc</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Ban Kỹ thuật</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/examhttps://drive.google.com/test-doc-x2https://drive.google.com/test-doc-x1ple-doc-123</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>⏳ Đang xử lý</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-07-24 14:30:46</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>